<commit_message>
Add Zanzibar hotel decision voting/comments and update itinerary spreadsheet
New "Zanzibar Hotel Decision" card in the Planning tab lists both booked
options (Hotel Riu Jambo, The Mora Zanzibar) with an upvote button and a
named comment thread per hotel, matching the existing Activity Wishlist
pattern. Flags the Sept 20th deadline to avoid losing the deposit.

Note: like the rest of the site's interactive features, votes/comments
are stored in localStorage (per device), not synced across everyone's
phones -- the card's disclaimer says so explicitly.

Also includes Carolyn's edits to Safari file.xlsx adding the two
Zanzibar hotel links to column E.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Safari file.xlsx
+++ b/Safari file.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carol\Dropbox\Family Room\2026 Safari Stonetown Tanzania\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carol\PycharmProjects\antigravity-experiments\Safari\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5EBF3C17-10B5-4320-B140-FAABBDD8E00C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9C4D252-96D5-4371-8178-D04D6BBEF5EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1CFB33F0-4E9F-40CD-8902-D633DCFD569E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="44">
   <si>
     <t>Sunday</t>
   </si>
@@ -137,13 +137,6 @@
     <t>Embalakai Authentic Camps https://share.google/WZiruAmUUqao5IlJW</t>
   </si>
   <si>
-    <t>To Serengeti
-Embalakai Authentic Camps</t>
-  </si>
-  <si>
-    <t>To Crater</t>
-  </si>
-  <si>
     <t>Ngorongoro Serena Safari Lodge https://share.google/TtoVYvMwfCVkwWey2</t>
   </si>
   <si>
@@ -182,15 +175,57 @@
     <t>https://share.google/aBPvUNMGdNFOjMAwT</t>
   </si>
   <si>
-    <t>After Tarangire NP
-Farm</t>
+    <t>To Crater Ngorongoro Serena Safari Lodge https://share.google/TtoVYvMwfCVkwWey2</t>
+  </si>
+  <si>
+    <t>To Serengeti https://share.google/WZiruAmUUqao5IlJW
+Embalakai Authentic Camps</t>
+  </si>
+  <si>
+    <t>To Crater, drive, https://share.google/468f4ixOubWuVeKMa
+Embalakai camp in Ngorongoro Camps</t>
+  </si>
+  <si>
+    <t>After Tarangire NP https://farmofdreamslodge.com/
+Farm of Dreams</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Fly to Kili transfer Arusha </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://www.serenahotels.com/arusha</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Serena Arusha</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">To Zanzibar Option 1 https://www.riu.com/en/hotel/tanzania/zanzibar/hotel-riu-jambo. Option 2 https://www.themora.com/zanzibar/ </t>
+  </si>
+  <si>
+    <t>Fly home</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -229,6 +264,13 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -626,7 +668,7 @@
         <v>9</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>10</v>
@@ -646,13 +688,13 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="70.5" x14ac:dyDescent="0.35">
@@ -666,19 +708,19 @@
         <v>16</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="84" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="98.5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -688,17 +730,17 @@
       <c r="C4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="70" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="84" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -712,16 +754,16 @@
         <v>12</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>24</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="70" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="84.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -731,17 +773,17 @@
       <c r="C6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="5" t="s">
         <v>12</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>24</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="70.5" x14ac:dyDescent="0.35">
@@ -758,14 +800,14 @@
         <v>13</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="70.5" x14ac:dyDescent="0.35">
@@ -782,14 +824,14 @@
         <v>13</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -806,7 +848,7 @@
         <v>14</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -819,6 +861,9 @@
       <c r="D10" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="E10" s="1" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
@@ -830,6 +875,9 @@
       <c r="D11" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="E11" s="1" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
@@ -841,6 +889,9 @@
       <c r="D12" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="E12" s="1" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
@@ -849,6 +900,9 @@
       <c r="B13" s="1">
         <v>3</v>
       </c>
+      <c r="E13" s="1" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
@@ -863,7 +917,7 @@
         <v>20</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
@@ -871,13 +925,15 @@
         <v>21</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D3" r:id="rId1" xr:uid="{EE7A4C91-94F2-4312-86CB-4D06FA25983F}"/>
+    <hyperlink ref="D6" r:id="rId2" xr:uid="{236B27F2-5BD0-4F02-A54B-7558B8352A42}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{483C09E6-4C1C-4C02-8A35-68A17104D6FC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>